<commit_message>
added pos and opp csvs
</commit_message>
<xml_diff>
--- a/Honors/statistic_id303555_us-per-capita-personal-income-by-state-2023 copy.xlsx
+++ b/Honors/statistic_id303555_us-per-capita-personal-income-by-state-2023 copy.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="11003"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sylviakniss/Documents/College/Senior Year 25/Hons 450/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sylviakniss/Documents/GitHub/knisssj/Honors/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D90BC8F-3797-5A4A-B7CC-929BF6659559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55B3E109-60C0-BF40-B2B3-D386F092EE2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="18900" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17600" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>

</xml_diff>